<commit_message>
Status of Funds: funding file (TDP, AFP, Reservations, Account) matched to the export by Functional Area (+ shared keys); Balance = TDP - Reservations - Obligation - Disbursement; funding.js module; realistic demo data; second List rows step in the flow; tests
</commit_message>
<xml_diff>
--- a/dashboards/finance/funds_template.xlsx
+++ b/dashboards/finance/funds_template.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Export" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Export" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -125,9 +125,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="FundsData" displayName="FundsData" ref="A1:I2" headerRowCount="1">
-  <autoFilter ref="A1:I2"/>
-  <tableColumns count="9">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="FundsData" displayName="FundsData" ref="A1:J2" headerRowCount="1">
+  <autoFilter ref="A1:J2"/>
+  <tableColumns count="10">
     <tableColumn id="1" name="contract_doc_no"/>
     <tableColumn id="2" name="commitment_item_fipex"/>
     <tableColumn id="3" name="functional_area_farea"/>
@@ -135,8 +135,9 @@
     <tableColumn id="5" name="fiscal_year"/>
     <tableColumn id="6" name="obligation_amt_cum"/>
     <tableColumn id="7" name="commitment_amt_cum"/>
-    <tableColumn id="8" name="sag"/>
-    <tableColumn id="9" name="mdep"/>
+    <tableColumn id="8" name="disbursement_amt_cum"/>
+    <tableColumn id="9" name="sag"/>
+    <tableColumn id="10" name="mdep"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
 </table>
@@ -431,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:J2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -443,6 +444,7 @@
     <col width="22" customWidth="1" min="7" max="7"/>
     <col width="22" customWidth="1" min="8" max="8"/>
     <col width="22" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -483,10 +485,15 @@
       </c>
       <c r="H1" t="inlineStr">
         <is>
+          <t>disbursement_amt_cum</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
           <t>sag</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>mdep</t>
         </is>

</xml_diff>